<commit_message>
Remove Captures sheet from spreadsheet — keep only sheets 1-4
User clarified they wanted to omit Captures and Notes, not Accounts.

https://claude.ai/code/session_0164EHQwJ8QsdKhyjAA5rh5F
</commit_message>
<xml_diff>
--- a/budget-manager.xlsx
+++ b/budget-manager.xlsx
@@ -13,7 +13,6 @@
     <sheet name="CC - JGW (9299)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="CC - SAMS (1261)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Bill Schedule" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Captures" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="WorkbenchBalance">Accounts!$B$13</definedName>
@@ -91,7 +90,7 @@
       <color rgb="0000B894"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -122,12 +121,6 @@
         <bgColor rgb="00D6DCE4"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4E6F1"/>
-        <bgColor rgb="00D4E6F1"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -147,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -190,10 +183,6 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1546,79 +1535,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="24" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="24" t="inlineStr">
-        <is>
-          <t>Projected Amount</t>
-        </is>
-      </c>
-      <c r="C1" s="24" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="21" t="n">
-        <v>46147</v>
-      </c>
-      <c r="B2" s="25" t="n">
-        <v>3245</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>After all May bills</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="21" t="n">
-        <v>46140</v>
-      </c>
-      <c r="B3" s="25" t="n">
-        <v>2100</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>After rent + utilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="21" t="n">
-        <v>46127</v>
-      </c>
-      <c r="B4" s="25" t="n">
-        <v>4800</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Post-paycheck snapshot</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>